<commit_message>
2nd and mens r16
</commit_message>
<xml_diff>
--- a/Knockouts/2ndAndBelow.xlsx
+++ b/Knockouts/2ndAndBelow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Ravens Seniors\Knockouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE700EF-57A6-4E00-AC43-C6BECBE9DAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A79AB5-D15B-4C37-8839-6185515393FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1" xr2:uid="{6F46E828-8FFD-4531-838C-1A16471CA10A}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="58">
   <si>
     <t>Match</t>
   </si>
@@ -230,6 +230,12 @@
   </si>
   <si>
     <t>Ilyaas Patel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>WO</t>
   </si>
 </sst>
 </file>
@@ -1505,7 +1511,7 @@
         <v xml:space="preserve">Boundary </v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G18" t="str" cm="1">
         <f t="array" ref="G18:I18">'Knockout Grid'!F8:H8</f>
@@ -1547,8 +1553,8 @@
       <c r="E19" t="str">
         <v>UCT</v>
       </c>
-      <c r="F19">
-        <v>0</v>
+      <c r="F19" t="str">
+        <v>WO</v>
       </c>
       <c r="G19" t="str" cm="1">
         <f t="array" ref="G19:I19">'Knockout Grid'!F16:H16</f>
@@ -1558,7 +1564,7 @@
         <v>Duinefontein TTC</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>25</v>
@@ -1591,7 +1597,7 @@
         <v>STEPH'S</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20" t="str" cm="1">
         <f t="array" ref="G20:I20">'Knockout Grid'!F24:H24</f>
@@ -1601,7 +1607,7 @@
         <v>Community House</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>25</v>
@@ -1634,7 +1640,7 @@
         <v>MP Royals</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G21" t="str" cm="1">
         <f t="array" ref="G21:I21">'Knockout Grid'!F32:H32</f>
@@ -1677,7 +1683,7 @@
         <v>Maties</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22" t="str" cm="1">
         <f t="array" ref="G22:I22">'Knockout Grid'!F40:H40</f>
@@ -1687,7 +1693,7 @@
         <v>Goodwood</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>25</v>
@@ -1720,7 +1726,7 @@
         <v>Mother City</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" t="str" cm="1">
         <f t="array" ref="G23:I23">'Knockout Grid'!F48:H48</f>
@@ -1730,7 +1736,7 @@
         <v>NEXUS</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>25</v>
@@ -1763,17 +1769,17 @@
         <v>NEXUS</v>
       </c>
       <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24" cm="1">
+        <v>3</v>
+      </c>
+      <c r="G24" t="str" cm="1">
         <f t="array" ref="G24:I24">'Knockout Grid'!F56:H56</f>
-        <v>0</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
+        <v>Allan Clark</v>
+      </c>
+      <c r="H24" t="str">
+        <v>TOP</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>25</v>
@@ -1806,7 +1812,7 @@
         <v>Maties</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G25" t="str" cm="1">
         <f t="array" ref="G25:I25">'Knockout Grid'!F64:H64</f>
@@ -1841,22 +1847,22 @@
       <c r="C26" t="s">
         <v>9</v>
       </c>
-      <c r="D26" cm="1">
+      <c r="D26" t="str" cm="1">
         <f t="array" ref="D26:F26">'Knockout Grid'!K11:M11</f>
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
+        <v>Musfiquh Kalam</v>
+      </c>
+      <c r="E26" t="str">
+        <v xml:space="preserve">Boundary </v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
-      <c r="G26" cm="1">
+      <c r="G26" t="str" cm="1">
         <f t="array" ref="G26:I26">'Knockout Grid'!K12:M12</f>
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>0</v>
+        <v>Adam Domingo</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Duinefontein TTC</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -1884,22 +1890,22 @@
       <c r="C27" t="s">
         <v>9</v>
       </c>
-      <c r="D27" cm="1">
+      <c r="D27" t="str" cm="1">
         <f t="array" ref="D27:F27">'Knockout Grid'!K27:M27</f>
-        <v>0</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
+        <v>Sedick Abrahams</v>
+      </c>
+      <c r="E27" t="str">
+        <v>STEPH'S</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
-      <c r="G27" cm="1">
+      <c r="G27" t="str" cm="1">
         <f t="array" ref="G27:I27">'Knockout Grid'!K28:M28</f>
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
+        <v>Ilyaas Patel</v>
+      </c>
+      <c r="H27" t="str">
+        <v>MP Royals</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -1927,22 +1933,22 @@
       <c r="C28" t="s">
         <v>9</v>
       </c>
-      <c r="D28" cm="1">
+      <c r="D28" t="str" cm="1">
         <f t="array" ref="D28:F28">'Knockout Grid'!K43:M43</f>
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>0</v>
+        <v>Tian Louw</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Maties</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
-      <c r="G28" cm="1">
+      <c r="G28" t="str" cm="1">
         <f t="array" ref="G28:I28">'Knockout Grid'!K44:M44</f>
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
+        <v>Amien Phillips</v>
+      </c>
+      <c r="H28" t="str">
+        <v>NEXUS</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1970,22 +1976,22 @@
       <c r="C29" t="s">
         <v>9</v>
       </c>
-      <c r="D29" cm="1">
+      <c r="D29" t="str" cm="1">
         <f t="array" ref="D29:F29">'Knockout Grid'!K59:M59</f>
-        <v>0</v>
-      </c>
-      <c r="E29">
-        <v>0</v>
+        <v>Craig Fortuin</v>
+      </c>
+      <c r="E29" t="str">
+        <v>NEXUS</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
-      <c r="G29" cm="1">
+      <c r="G29" t="str" cm="1">
         <f t="array" ref="G29:I29">'Knockout Grid'!K60:M60</f>
-        <v>0</v>
-      </c>
-      <c r="H29">
-        <v>0</v>
+        <v>DJ Swanevelder</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Maties</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -2320,7 +2326,9 @@
       <c r="G7" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="10">
+        <v>3</v>
+      </c>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
@@ -2340,7 +2348,9 @@
       <c r="G8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="10">
+        <v>0</v>
+      </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -2386,8 +2396,12 @@
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="I11" s="4"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="9"/>
+      <c r="K11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>47</v>
+      </c>
       <c r="M11" s="10"/>
       <c r="N11" s="2"/>
     </row>
@@ -2402,8 +2416,12 @@
         <v>3</v>
       </c>
       <c r="I12" s="4"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="9"/>
+      <c r="K12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>44</v>
+      </c>
       <c r="M12" s="10"/>
       <c r="N12" s="1"/>
     </row>
@@ -2458,7 +2476,9 @@
       <c r="G15" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="H15" s="10"/>
+      <c r="H15" s="10" t="s">
+        <v>57</v>
+      </c>
       <c r="I15" s="5"/>
       <c r="N15" s="4"/>
     </row>
@@ -2479,7 +2499,9 @@
       <c r="G16" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="H16" s="10"/>
+      <c r="H16" s="10">
+        <v>3</v>
+      </c>
       <c r="N16" s="4"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -2610,7 +2632,9 @@
       <c r="G23" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H23" s="10"/>
+      <c r="H23" s="10">
+        <v>3</v>
+      </c>
       <c r="I23" s="2"/>
       <c r="N23" s="4"/>
       <c r="S23" s="4"/>
@@ -2632,7 +2656,9 @@
       <c r="G24" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="H24" s="10"/>
+      <c r="H24" s="10">
+        <v>1</v>
+      </c>
       <c r="I24" s="1"/>
       <c r="N24" s="4"/>
       <c r="S24" s="4"/>
@@ -2690,8 +2716,12 @@
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="I27" s="4"/>
       <c r="J27" s="2"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="9"/>
+      <c r="K27" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L27" s="9" t="s">
+        <v>38</v>
+      </c>
       <c r="M27" s="10"/>
       <c r="N27" s="5"/>
       <c r="S27" s="4"/>
@@ -2707,8 +2737,12 @@
         <v>7</v>
       </c>
       <c r="I28" s="4"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="9"/>
+      <c r="K28" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="L28" s="9" t="s">
+        <v>32</v>
+      </c>
       <c r="M28" s="10"/>
       <c r="S28" s="4"/>
     </row>
@@ -2764,7 +2798,9 @@
       <c r="G31" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H31" s="10"/>
+      <c r="H31" s="10">
+        <v>3</v>
+      </c>
       <c r="I31" s="5"/>
       <c r="S31" s="4"/>
     </row>
@@ -2785,7 +2821,9 @@
       <c r="G32" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="H32" s="10"/>
+      <c r="H32" s="10">
+        <v>0</v>
+      </c>
       <c r="S32" s="4"/>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.25">
@@ -2892,7 +2930,9 @@
       <c r="G39" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="H39" s="10"/>
+      <c r="H39" s="10">
+        <v>3</v>
+      </c>
       <c r="I39" s="2"/>
       <c r="S39" s="4"/>
     </row>
@@ -2913,7 +2953,9 @@
       <c r="G40" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="H40" s="10"/>
+      <c r="H40" s="10">
+        <v>1</v>
+      </c>
       <c r="I40" s="1"/>
       <c r="S40" s="4"/>
     </row>
@@ -2974,8 +3016,12 @@
       </c>
       <c r="I43" s="4"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="8"/>
-      <c r="L43" s="9"/>
+      <c r="K43" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="L43" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="M43" s="10"/>
       <c r="N43" s="2"/>
       <c r="S43" s="4"/>
@@ -2990,9 +3036,16 @@
       <c r="C44">
         <v>11</v>
       </c>
+      <c r="F44" t="s">
+        <v>56</v>
+      </c>
       <c r="I44" s="4"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="9"/>
+      <c r="K44" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="M44" s="10"/>
       <c r="N44" s="1"/>
       <c r="S44" s="4"/>
@@ -3057,7 +3110,9 @@
       <c r="G47" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="H47" s="10"/>
+      <c r="H47" s="10">
+        <v>2</v>
+      </c>
       <c r="I47" s="5"/>
       <c r="N47" s="4"/>
       <c r="S47" s="4"/>
@@ -3079,7 +3134,9 @@
       <c r="G48" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="H48" s="10"/>
+      <c r="H48" s="10">
+        <v>3</v>
+      </c>
       <c r="N48" s="4"/>
       <c r="S48" s="4"/>
     </row>
@@ -3189,7 +3246,9 @@
       <c r="G55" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="H55" s="10"/>
+      <c r="H55" s="10">
+        <v>3</v>
+      </c>
       <c r="I55" s="2"/>
       <c r="N55" s="4"/>
     </row>
@@ -3204,9 +3263,15 @@
         <v>14</v>
       </c>
       <c r="D56" s="4"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="10"/>
+      <c r="F56" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G56" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H56" s="10">
+        <v>1</v>
+      </c>
       <c r="I56" s="1"/>
       <c r="N56" s="4"/>
     </row>
@@ -3255,8 +3320,12 @@
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="I59" s="4"/>
       <c r="J59" s="2"/>
-      <c r="K59" s="8"/>
-      <c r="L59" s="9"/>
+      <c r="K59" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L59" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="M59" s="10"/>
       <c r="N59" s="5"/>
     </row>
@@ -3271,8 +3340,12 @@
         <v>15</v>
       </c>
       <c r="I60" s="4"/>
-      <c r="K60" s="8"/>
-      <c r="L60" s="9"/>
+      <c r="K60" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="L60" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="M60" s="10"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
@@ -3324,7 +3397,9 @@
       <c r="G63" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="H63" s="10"/>
+      <c r="H63" s="10">
+        <v>3</v>
+      </c>
       <c r="I63" s="5"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
@@ -3344,7 +3419,9 @@
       <c r="G64" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="H64" s="10"/>
+      <c r="H64" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">

</xml_diff>

<commit_message>
Mens and 2nd Below semis
</commit_message>
<xml_diff>
--- a/Knockouts/2ndAndBelow.xlsx
+++ b/Knockouts/2ndAndBelow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Ravens Seniors\Knockouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAD0D5A-3AB9-456A-A693-CBF4B4356045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B66D3A68-B3FB-4B7F-9CDB-324FCE7AF127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1" xr2:uid="{6F46E828-8FFD-4531-838C-1A16471CA10A}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="58">
   <si>
     <t>Match</t>
   </si>
@@ -2027,7 +2027,7 @@
         <v xml:space="preserve">Boundary </v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G30" t="str" cm="1">
         <f t="array" ref="G30:I30">'Knockout Grid'!P20:R20</f>
@@ -2070,7 +2070,7 @@
         <v>Maties</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" t="str" cm="1">
         <f t="array" ref="G31:I31">'Knockout Grid'!P52:R52</f>
@@ -2080,7 +2080,7 @@
         <v>Maties</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>25</v>
@@ -2105,22 +2105,22 @@
       <c r="C32" t="s">
         <v>11</v>
       </c>
-      <c r="D32" cm="1">
+      <c r="D32" t="str" cm="1">
         <f t="array" ref="D32:F32">'Knockout Grid'!U35:W35</f>
-        <v>0</v>
-      </c>
-      <c r="E32">
-        <v>0</v>
+        <v>Musfiquh Kalam</v>
+      </c>
+      <c r="E32" t="str">
+        <v xml:space="preserve">Boundary </v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
-      <c r="G32" cm="1">
+      <c r="G32" t="str" cm="1">
         <f t="array" ref="G32:I32">'Knockout Grid'!U36:W36</f>
-        <v>0</v>
-      </c>
-      <c r="H32">
-        <v>0</v>
+        <v>Tian Louw</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Maties</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -2557,7 +2557,9 @@
       <c r="Q19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="R19" s="10"/>
+      <c r="R19" s="10">
+        <v>3</v>
+      </c>
       <c r="S19" s="2"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -2577,7 +2579,9 @@
       <c r="Q20" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="R20" s="10"/>
+      <c r="R20" s="10">
+        <v>0</v>
+      </c>
       <c r="S20" s="1"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -2876,8 +2880,12 @@
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="S35" s="4"/>
       <c r="T35" s="2"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="9"/>
+      <c r="U35" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="V35" s="9" t="s">
+        <v>47</v>
+      </c>
       <c r="W35" s="10"/>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
@@ -2891,8 +2899,12 @@
         <v>9</v>
       </c>
       <c r="S36" s="4"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="9"/>
+      <c r="U36" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="V36" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="W36" s="10"/>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
@@ -3201,7 +3213,9 @@
       <c r="Q51" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="R51" s="10"/>
+      <c r="R51" s="10">
+        <v>3</v>
+      </c>
       <c r="S51" s="5"/>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
@@ -3221,7 +3235,9 @@
       <c r="Q52" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="R52" s="10"/>
+      <c r="R52" s="10">
+        <v>2</v>
+      </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">

</xml_diff>

<commit_message>
Mens final and 2nd final
</commit_message>
<xml_diff>
--- a/Knockouts/2ndAndBelow.xlsx
+++ b/Knockouts/2ndAndBelow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Ravens Seniors\Knockouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B66D3A68-B3FB-4B7F-9CDB-324FCE7AF127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C3A23A-9CC1-4F0C-8B0D-9011CD3F43D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1" xr2:uid="{6F46E828-8FFD-4531-838C-1A16471CA10A}"/>
   </bookViews>
@@ -2113,7 +2113,7 @@
         <v xml:space="preserve">Boundary </v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" t="str" cm="1">
         <f t="array" ref="G32:I32">'Knockout Grid'!U36:W36</f>
@@ -2123,7 +2123,7 @@
         <v>Maties</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>25</v>
@@ -2886,7 +2886,9 @@
       <c r="V35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="W35" s="10"/>
+      <c r="W35" s="10">
+        <v>2</v>
+      </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
@@ -2905,7 +2907,9 @@
       <c r="V36" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="W36" s="10"/>
+      <c r="W36" s="10">
+        <v>3</v>
+      </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">

</xml_diff>